<commit_message>
Add plan for Limited Company (March Year-End) package generation
</commit_message>
<xml_diff>
--- a/packages/GB Accounts Self Employed 2023-04-05 (Apr23) Excel 2007/Salesinvoice.xlsx
+++ b/packages/GB Accounts Self Employed 2023-04-05 (Apr23) Excel 2007/Salesinvoice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10311"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\louis\Downloads\Packages to create\GB Accounts Company 2022-03-31 (Mar22) Excel 2007\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antony/projects/diy-accounting/GB Accounts 2024-25/GB Accounts Invoice Generator 2025-12-31 (Dec25) Excel 2007/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA93E1E-4C50-4676-8B3C-77CC8AD343F9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18417B1-DFBF-A440-B42A-AAB3CE6305FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="724" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="23640" windowHeight="17940" tabRatio="724" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice Template" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Avoid typing directly into the "Invoice Template" sheet - all customer and product data should be pulled from the Customer and Product Details sheets.</t>
         </r>
@@ -492,13 +492,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="8" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
-    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="0.00_ ;[Red]\-0.00\ "/>
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00_ ;[Red]\-#,##0.00\ "/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0.00_ ;[Red]\-0.00\ "/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -506,6 +506,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -610,12 +611,6 @@
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -991,13 +986,13 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="8" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1012,13 +1007,13 @@
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
@@ -1037,10 +1032,10 @@
     <xf numFmtId="1" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1050,8 +1045,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1077,7 +1072,7 @@
     <xf numFmtId="4" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="20" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1085,7 +1080,7 @@
     <xf numFmtId="4" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="20" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1096,36 +1091,36 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
     <xf numFmtId="4" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="20" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="20" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="20" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="19" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1134,15 +1129,138 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1154,129 +1272,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="8" fontId="9" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1303,9 +1298,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1343,9 +1338,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1378,26 +1373,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1430,26 +1408,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1627,31 +1588,31 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V70"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="2.140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="3.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="0.85546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="2.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="3.1640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="0.83203125" style="2" customWidth="1"/>
     <col min="5" max="7" width="9" style="2" customWidth="1"/>
-    <col min="8" max="8" width="6.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="0.85546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="6.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="0.83203125" style="2" customWidth="1"/>
     <col min="10" max="10" width="9" style="2" customWidth="1"/>
-    <col min="11" max="11" width="0.85546875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" style="2" customWidth="1"/>
-    <col min="13" max="13" width="0.85546875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="9.7109375" style="2" customWidth="1"/>
-    <col min="15" max="15" width="0.85546875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="12.5703125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="0.85546875" style="2" customWidth="1"/>
-    <col min="18" max="18" width="3.28515625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="2.140625" style="2" customWidth="1"/>
-    <col min="20" max="21" width="9.140625" style="2"/>
-    <col min="22" max="22" width="9.140625" style="61" hidden="1" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="2"/>
+    <col min="11" max="11" width="0.83203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="9.6640625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="0.83203125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="9.6640625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="0.83203125" style="2" customWidth="1"/>
+    <col min="16" max="16" width="12.5" style="2" customWidth="1"/>
+    <col min="17" max="17" width="0.83203125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="3.33203125" style="2" customWidth="1"/>
+    <col min="19" max="19" width="2.1640625" style="2" customWidth="1"/>
+    <col min="20" max="21" width="9.1640625" style="2"/>
+    <col min="22" max="22" width="9.1640625" style="61" hidden="1" customWidth="1"/>
+    <col min="23" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="12" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1674,13 +1635,13 @@
     </row>
     <row r="2" spans="1:19" ht="7.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1"/>
-      <c r="G2" s="105" t="s">
+      <c r="G2" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="106"/>
-      <c r="I2" s="106"/>
-      <c r="J2" s="106"/>
-      <c r="K2" s="107"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="76"/>
+      <c r="J2" s="76"/>
+      <c r="K2" s="77"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -1692,11 +1653,11 @@
     </row>
     <row r="3" spans="1:19" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
-      <c r="G3" s="108"/>
-      <c r="H3" s="109"/>
-      <c r="I3" s="109"/>
-      <c r="J3" s="109"/>
-      <c r="K3" s="110"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="80"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -1718,14 +1679,14 @@
     </row>
     <row r="5" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1"/>
-      <c r="C5" s="87" t="str">
+      <c r="C5" s="118" t="str">
         <f>IF('Business Details'!B2&gt;0,'Business Details'!B2," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="D5" s="87"/>
-      <c r="E5" s="87"/>
-      <c r="F5" s="87"/>
-      <c r="G5" s="87"/>
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
+      <c r="G5" s="118"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -1735,26 +1696,26 @@
     </row>
     <row r="6" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1"/>
-      <c r="C6" s="87"/>
-      <c r="D6" s="87"/>
-      <c r="E6" s="87"/>
-      <c r="F6" s="87"/>
-      <c r="G6" s="87"/>
-      <c r="J6" s="83" t="str">
+      <c r="C6" s="118"/>
+      <c r="D6" s="118"/>
+      <c r="E6" s="118"/>
+      <c r="F6" s="118"/>
+      <c r="G6" s="118"/>
+      <c r="J6" s="113" t="str">
         <f>IF('Business Details'!B12&gt;0,'Business Details'!B12," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K6" s="83"/>
-      <c r="L6" s="83"/>
-      <c r="M6" s="83"/>
-      <c r="N6" s="83"/>
-      <c r="O6" s="83"/>
-      <c r="P6" s="83"/>
+      <c r="K6" s="113"/>
+      <c r="L6" s="113"/>
+      <c r="M6" s="113"/>
+      <c r="N6" s="113"/>
+      <c r="O6" s="113"/>
+      <c r="P6" s="113"/>
       <c r="Q6" s="13"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -1774,27 +1735,27 @@
     </row>
     <row r="8" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1"/>
-      <c r="C8" s="82" t="str">
+      <c r="C8" s="114" t="str">
         <f>IF('Business Details'!B13&gt;0,'Business Details'!B13," ")</f>
         <v>Thank you for your custom</v>
       </c>
-      <c r="D8" s="82"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
-      <c r="J8" s="122" t="str">
+      <c r="D8" s="114"/>
+      <c r="E8" s="114"/>
+      <c r="F8" s="114"/>
+      <c r="G8" s="114"/>
+      <c r="J8" s="98" t="str">
         <f>IF(O8=" "," ",'Business Details'!A11)</f>
         <v>VAT Registration Number</v>
       </c>
-      <c r="K8" s="122"/>
-      <c r="L8" s="122"/>
-      <c r="M8" s="122"/>
-      <c r="N8" s="122"/>
-      <c r="O8" s="119" t="str">
+      <c r="K8" s="98"/>
+      <c r="L8" s="98"/>
+      <c r="M8" s="98"/>
+      <c r="N8" s="98"/>
+      <c r="O8" s="94" t="str">
         <f>IF('Business Details'!B11&gt;0,'Business Details'!B11," ")</f>
         <v xml:space="preserve">  </v>
       </c>
-      <c r="P8" s="120"/>
+      <c r="P8" s="95"/>
       <c r="Q8" s="11"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
@@ -1806,25 +1767,25 @@
     </row>
     <row r="10" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1"/>
-      <c r="C10" s="84" t="s">
+      <c r="C10" s="115" t="s">
         <v>74</v>
       </c>
-      <c r="D10" s="85"/>
-      <c r="E10" s="85"/>
-      <c r="F10" s="85"/>
-      <c r="G10" s="86"/>
+      <c r="D10" s="116"/>
+      <c r="E10" s="116"/>
+      <c r="F10" s="116"/>
+      <c r="G10" s="117"/>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
-      <c r="J10" s="121" t="str">
+      <c r="J10" s="96" t="str">
         <f>IF('Business Details'!B3&gt;0,'Business Details'!B3," ")</f>
         <v>&lt;enter business name&gt;</v>
       </c>
-      <c r="K10" s="121"/>
-      <c r="L10" s="121"/>
-      <c r="M10" s="121"/>
-      <c r="N10" s="121"/>
-      <c r="O10" s="121"/>
-      <c r="P10" s="121"/>
+      <c r="K10" s="96"/>
+      <c r="L10" s="96"/>
+      <c r="M10" s="96"/>
+      <c r="N10" s="96"/>
+      <c r="O10" s="96"/>
+      <c r="P10" s="96"/>
       <c r="Q10" s="7"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
@@ -1838,13 +1799,13 @@
       <c r="G11" s="6"/>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
-      <c r="J11" s="121"/>
-      <c r="K11" s="121"/>
-      <c r="L11" s="121"/>
-      <c r="M11" s="121"/>
-      <c r="N11" s="121"/>
-      <c r="O11" s="121"/>
-      <c r="P11" s="121"/>
+      <c r="J11" s="96"/>
+      <c r="K11" s="96"/>
+      <c r="L11" s="96"/>
+      <c r="M11" s="96"/>
+      <c r="N11" s="96"/>
+      <c r="O11" s="96"/>
+      <c r="P11" s="96"/>
       <c r="Q11" s="7"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
@@ -1861,16 +1822,16 @@
       <c r="G12" s="74"/>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
-      <c r="J12" s="75" t="str">
+      <c r="J12" s="97" t="str">
         <f>IF('Business Details'!B4&gt;0,'Business Details'!B4," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K12" s="75"/>
-      <c r="L12" s="75"/>
-      <c r="M12" s="75"/>
-      <c r="N12" s="75"/>
-      <c r="O12" s="75"/>
-      <c r="P12" s="75"/>
+      <c r="K12" s="97"/>
+      <c r="L12" s="97"/>
+      <c r="M12" s="97"/>
+      <c r="N12" s="97"/>
+      <c r="O12" s="97"/>
+      <c r="P12" s="97"/>
       <c r="Q12" s="7"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -1884,13 +1845,13 @@
       <c r="G13" s="74"/>
       <c r="H13" s="7"/>
       <c r="I13" s="7"/>
-      <c r="J13" s="75"/>
-      <c r="K13" s="75"/>
-      <c r="L13" s="75"/>
-      <c r="M13" s="75"/>
-      <c r="N13" s="75"/>
-      <c r="O13" s="75"/>
-      <c r="P13" s="75"/>
+      <c r="J13" s="97"/>
+      <c r="K13" s="97"/>
+      <c r="L13" s="97"/>
+      <c r="M13" s="97"/>
+      <c r="N13" s="97"/>
+      <c r="O13" s="97"/>
+      <c r="P13" s="97"/>
       <c r="Q13" s="7"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
@@ -1907,16 +1868,16 @@
       <c r="G14" s="74"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
-      <c r="J14" s="75" t="str">
+      <c r="J14" s="97" t="str">
         <f>IF('Business Details'!B5&gt;0,'Business Details'!B5," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K14" s="75"/>
-      <c r="L14" s="75"/>
-      <c r="M14" s="75"/>
-      <c r="N14" s="75"/>
-      <c r="O14" s="75"/>
-      <c r="P14" s="75"/>
+      <c r="K14" s="97"/>
+      <c r="L14" s="97"/>
+      <c r="M14" s="97"/>
+      <c r="N14" s="97"/>
+      <c r="O14" s="97"/>
+      <c r="P14" s="97"/>
       <c r="Q14" s="7"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
@@ -1930,13 +1891,13 @@
       <c r="G15" s="74"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
-      <c r="J15" s="75"/>
-      <c r="K15" s="75"/>
-      <c r="L15" s="75"/>
-      <c r="M15" s="75"/>
-      <c r="N15" s="75"/>
-      <c r="O15" s="75"/>
-      <c r="P15" s="75"/>
+      <c r="J15" s="97"/>
+      <c r="K15" s="97"/>
+      <c r="L15" s="97"/>
+      <c r="M15" s="97"/>
+      <c r="N15" s="97"/>
+      <c r="O15" s="97"/>
+      <c r="P15" s="97"/>
       <c r="Q15" s="7"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
@@ -1953,16 +1914,16 @@
       <c r="G16" s="74"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="75" t="str">
+      <c r="J16" s="97" t="str">
         <f>IF('Business Details'!B6&gt;0,'Business Details'!B6," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K16" s="75"/>
-      <c r="L16" s="75"/>
-      <c r="M16" s="75"/>
-      <c r="N16" s="75"/>
-      <c r="O16" s="75"/>
-      <c r="P16" s="75"/>
+      <c r="K16" s="97"/>
+      <c r="L16" s="97"/>
+      <c r="M16" s="97"/>
+      <c r="N16" s="97"/>
+      <c r="O16" s="97"/>
+      <c r="P16" s="97"/>
       <c r="Q16" s="7"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
@@ -1976,13 +1937,13 @@
       <c r="G17" s="74"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7"/>
-      <c r="J17" s="75"/>
-      <c r="K17" s="75"/>
-      <c r="L17" s="75"/>
-      <c r="M17" s="75"/>
-      <c r="N17" s="75"/>
-      <c r="O17" s="75"/>
-      <c r="P17" s="75"/>
+      <c r="J17" s="97"/>
+      <c r="K17" s="97"/>
+      <c r="L17" s="97"/>
+      <c r="M17" s="97"/>
+      <c r="N17" s="97"/>
+      <c r="O17" s="97"/>
+      <c r="P17" s="97"/>
       <c r="Q17" s="7"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
@@ -1999,16 +1960,16 @@
       <c r="G18" s="74"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7"/>
-      <c r="J18" s="75" t="str">
+      <c r="J18" s="97" t="str">
         <f>IF('Business Details'!B7&gt;0,'Business Details'!B7," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="K18" s="75"/>
-      <c r="L18" s="75"/>
-      <c r="M18" s="75"/>
-      <c r="N18" s="75"/>
-      <c r="O18" s="75"/>
-      <c r="P18" s="75"/>
+      <c r="K18" s="97"/>
+      <c r="L18" s="97"/>
+      <c r="M18" s="97"/>
+      <c r="N18" s="97"/>
+      <c r="O18" s="97"/>
+      <c r="P18" s="97"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -2022,13 +1983,13 @@
       <c r="G19" s="6"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7"/>
-      <c r="J19" s="92"/>
-      <c r="K19" s="92"/>
-      <c r="L19" s="92"/>
-      <c r="M19" s="92"/>
-      <c r="N19" s="92"/>
-      <c r="O19" s="92"/>
-      <c r="P19" s="92"/>
+      <c r="J19" s="81"/>
+      <c r="K19" s="81"/>
+      <c r="L19" s="81"/>
+      <c r="M19" s="81"/>
+      <c r="N19" s="81"/>
+      <c r="O19" s="81"/>
+      <c r="P19" s="81"/>
       <c r="Q19" s="7"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -2045,19 +2006,19 @@
       <c r="G20" s="74"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
-      <c r="J20" s="100" t="str">
+      <c r="J20" s="103" t="str">
         <f>'Business Details'!A8</f>
         <v>Telephone</v>
       </c>
-      <c r="K20" s="100"/>
-      <c r="L20" s="100"/>
+      <c r="K20" s="103"/>
+      <c r="L20" s="103"/>
       <c r="M20" s="10"/>
-      <c r="N20" s="101" t="str">
+      <c r="N20" s="87" t="str">
         <f>IF('Business Details'!B8&gt;0,'Business Details'!B8," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="O20" s="101"/>
-      <c r="P20" s="101"/>
+      <c r="O20" s="87"/>
+      <c r="P20" s="87"/>
       <c r="Q20" s="7"/>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
@@ -2071,13 +2032,13 @@
       <c r="G21" s="6"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7"/>
-      <c r="J21" s="99"/>
-      <c r="K21" s="99"/>
-      <c r="L21" s="99"/>
-      <c r="M21" s="99"/>
-      <c r="N21" s="99"/>
-      <c r="O21" s="99"/>
-      <c r="P21" s="99"/>
+      <c r="J21" s="102"/>
+      <c r="K21" s="102"/>
+      <c r="L21" s="102"/>
+      <c r="M21" s="102"/>
+      <c r="N21" s="102"/>
+      <c r="O21" s="102"/>
+      <c r="P21" s="102"/>
       <c r="Q21" s="7"/>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
@@ -2091,19 +2052,19 @@
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
       <c r="I22" s="7"/>
-      <c r="J22" s="100" t="str">
+      <c r="J22" s="103" t="str">
         <f>'Business Details'!A9</f>
         <v>Fax number</v>
       </c>
-      <c r="K22" s="100"/>
-      <c r="L22" s="100"/>
+      <c r="K22" s="103"/>
+      <c r="L22" s="103"/>
       <c r="M22" s="10"/>
-      <c r="N22" s="101" t="str">
+      <c r="N22" s="87" t="str">
         <f>IF('Business Details'!B9&gt;0,'Business Details'!B9," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="O22" s="101"/>
-      <c r="P22" s="101"/>
+      <c r="O22" s="87"/>
+      <c r="P22" s="87"/>
       <c r="Q22" s="7"/>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
@@ -2117,13 +2078,13 @@
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
       <c r="I23" s="7"/>
-      <c r="J23" s="99"/>
-      <c r="K23" s="99"/>
-      <c r="L23" s="99"/>
-      <c r="M23" s="99"/>
-      <c r="N23" s="99"/>
-      <c r="O23" s="99"/>
-      <c r="P23" s="99"/>
+      <c r="J23" s="102"/>
+      <c r="K23" s="102"/>
+      <c r="L23" s="102"/>
+      <c r="M23" s="102"/>
+      <c r="N23" s="102"/>
+      <c r="O23" s="102"/>
+      <c r="P23" s="102"/>
       <c r="Q23" s="7"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
@@ -2135,30 +2096,30 @@
         <v xml:space="preserve">Email </v>
       </c>
       <c r="K24" s="15"/>
-      <c r="L24" s="116" t="str">
+      <c r="L24" s="90" t="str">
         <f>IF('Business Details'!B10&gt;0,'Business Details'!B10," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="M24" s="117"/>
-      <c r="N24" s="117"/>
-      <c r="O24" s="117"/>
-      <c r="P24" s="117"/>
+      <c r="M24" s="91"/>
+      <c r="N24" s="91"/>
+      <c r="O24" s="91"/>
+      <c r="P24" s="91"/>
       <c r="Q24" s="7"/>
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
     </row>
     <row r="25" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="1"/>
-      <c r="C25" s="84" t="s">
+      <c r="C25" s="115" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="85"/>
-      <c r="E25" s="85"/>
-      <c r="F25" s="85"/>
-      <c r="G25" s="86"/>
-      <c r="N25" s="118"/>
-      <c r="O25" s="118"/>
-      <c r="P25" s="118"/>
+      <c r="D25" s="116"/>
+      <c r="E25" s="116"/>
+      <c r="F25" s="116"/>
+      <c r="G25" s="117"/>
+      <c r="N25" s="92"/>
+      <c r="O25" s="92"/>
+      <c r="P25" s="92"/>
       <c r="Q25" s="3"/>
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
@@ -2170,9 +2131,9 @@
       <c r="E26" s="74"/>
       <c r="F26" s="74"/>
       <c r="G26" s="74"/>
-      <c r="N26" s="118"/>
-      <c r="O26" s="118"/>
-      <c r="P26" s="118"/>
+      <c r="N26" s="92"/>
+      <c r="O26" s="92"/>
+      <c r="P26" s="92"/>
       <c r="Q26" s="3"/>
       <c r="R26" s="1"/>
       <c r="S26" s="1"/>
@@ -2187,18 +2148,18 @@
       <c r="E27" s="74"/>
       <c r="F27" s="74"/>
       <c r="G27" s="74"/>
-      <c r="J27" s="102" t="s">
-        <v>20</v>
-      </c>
-      <c r="K27" s="102"/>
-      <c r="L27" s="102"/>
+      <c r="J27" s="93" t="s">
+        <v>20</v>
+      </c>
+      <c r="K27" s="93"/>
+      <c r="L27" s="93"/>
       <c r="M27" s="7"/>
-      <c r="N27" s="111" t="str">
+      <c r="N27" s="84" t="str">
         <f>IF(SUM('Invoice Database'!A:A)=0," ",LOOKUP(1,'Invoice Database'!A:A,'Invoice Database'!B:B))</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="O27" s="112"/>
-      <c r="P27" s="113"/>
+      <c r="O27" s="85"/>
+      <c r="P27" s="86"/>
       <c r="Q27" s="7"/>
       <c r="R27" s="1"/>
       <c r="S27" s="1"/>
@@ -2231,18 +2192,18 @@
       <c r="E29" s="74"/>
       <c r="F29" s="74"/>
       <c r="G29" s="74"/>
-      <c r="J29" s="102" t="s">
+      <c r="J29" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="102"/>
-      <c r="L29" s="102"/>
+      <c r="K29" s="93"/>
+      <c r="L29" s="93"/>
       <c r="M29" s="7"/>
-      <c r="N29" s="111" t="str">
+      <c r="N29" s="84" t="str">
         <f>IF(N27=" "," ",IF(N27&gt;0,LOOKUP(N27,'Invoice Database'!B:B,'Invoice Database'!D:D)))</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="O29" s="112"/>
-      <c r="P29" s="113"/>
+      <c r="O29" s="85"/>
+      <c r="P29" s="86"/>
       <c r="Q29" s="7"/>
       <c r="R29" s="1"/>
       <c r="S29" s="1"/>
@@ -2275,18 +2236,18 @@
       <c r="E31" s="74"/>
       <c r="F31" s="74"/>
       <c r="G31" s="74"/>
-      <c r="J31" s="102" t="s">
+      <c r="J31" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="K31" s="102"/>
-      <c r="L31" s="102"/>
+      <c r="K31" s="93"/>
+      <c r="L31" s="93"/>
       <c r="M31" s="7"/>
-      <c r="N31" s="111" t="str">
+      <c r="N31" s="84" t="str">
         <f>IF(N27=" "," ",IF(N27&gt;0,LOOKUP(N29,'Customer Details'!A:A,'Customer Details'!B:B)))</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="O31" s="112"/>
-      <c r="P31" s="113"/>
+      <c r="O31" s="85"/>
+      <c r="P31" s="86"/>
       <c r="Q31" s="7"/>
       <c r="R31" s="1"/>
       <c r="S31" s="1"/>
@@ -2325,12 +2286,12 @@
       <c r="K33" s="74"/>
       <c r="L33" s="74"/>
       <c r="M33" s="7"/>
-      <c r="N33" s="114" t="str">
+      <c r="N33" s="88" t="str">
         <f>IF(N27=" "," ",IF(N27&gt;0,LOOKUP(N27,'Invoice Database'!B:B,'Invoice Database'!C:C)))</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="O33" s="115"/>
-      <c r="P33" s="113"/>
+      <c r="O33" s="89"/>
+      <c r="P33" s="86"/>
       <c r="Q33" s="7"/>
       <c r="R33" s="1"/>
       <c r="S33" s="1"/>
@@ -2365,19 +2326,19 @@
       <c r="R36" s="1"/>
       <c r="S36" s="1"/>
     </row>
-    <row r="37" spans="1:22" ht="22.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:22" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="33" t="s">
         <v>6</v>
       </c>
       <c r="D37" s="34"/>
-      <c r="E37" s="80" t="s">
+      <c r="E37" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="F37" s="81"/>
-      <c r="G37" s="81"/>
-      <c r="H37" s="81"/>
+      <c r="F37" s="122"/>
+      <c r="G37" s="122"/>
+      <c r="H37" s="122"/>
       <c r="I37" s="34"/>
       <c r="J37" s="33" t="s">
         <v>24</v>
@@ -2391,10 +2352,10 @@
         <v>28</v>
       </c>
       <c r="O37" s="34"/>
-      <c r="P37" s="78" t="s">
+      <c r="P37" s="119" t="s">
         <v>27</v>
       </c>
-      <c r="Q37" s="79"/>
+      <c r="Q37" s="120"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
     </row>
@@ -2429,11 +2390,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O38" s="28"/>
-      <c r="P38" s="76" t="str">
+      <c r="P38" s="106" t="str">
         <f>IF(L38=" "," ",J38*L38)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q38" s="77"/>
+      <c r="Q38" s="107"/>
       <c r="R38" s="1"/>
       <c r="S38" s="1"/>
       <c r="V38" s="61">
@@ -2472,11 +2433,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O39" s="28"/>
-      <c r="P39" s="76" t="str">
+      <c r="P39" s="106" t="str">
         <f>IF(L39=" "," ",J39*L39)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q39" s="77"/>
+      <c r="Q39" s="107"/>
       <c r="R39" s="1"/>
       <c r="S39" s="1"/>
       <c r="V39" s="61">
@@ -2515,11 +2476,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O40" s="28"/>
-      <c r="P40" s="76" t="str">
+      <c r="P40" s="106" t="str">
         <f>IF(L40=" "," ",J40*L40)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q40" s="77"/>
+      <c r="Q40" s="107"/>
       <c r="R40" s="1"/>
       <c r="S40" s="1"/>
       <c r="V40" s="61">
@@ -2558,11 +2519,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O41" s="28"/>
-      <c r="P41" s="76" t="str">
+      <c r="P41" s="106" t="str">
         <f>IF(L41=" "," ",J41*L41)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q41" s="77"/>
+      <c r="Q41" s="107"/>
       <c r="R41" s="1"/>
       <c r="S41" s="1"/>
       <c r="U41" s="31"/>
@@ -2602,11 +2563,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O42" s="28"/>
-      <c r="P42" s="76" t="str">
+      <c r="P42" s="106" t="str">
         <f>IF(L42=" "," ",J42*L42)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q42" s="77"/>
+      <c r="Q42" s="107"/>
       <c r="R42" s="1"/>
       <c r="S42" s="1"/>
       <c r="V42" s="61">
@@ -2645,11 +2606,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O43" s="28"/>
-      <c r="P43" s="76" t="str">
+      <c r="P43" s="106" t="str">
         <f t="shared" ref="P43:P57" si="1">IF(L43=" "," ",J43*L43)</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q43" s="77"/>
+      <c r="Q43" s="107"/>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
       <c r="V43" s="61">
@@ -2688,11 +2649,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O44" s="28"/>
-      <c r="P44" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q44" s="77"/>
+      <c r="P44" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q44" s="107"/>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
       <c r="V44" s="61">
@@ -2731,11 +2692,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O45" s="28"/>
-      <c r="P45" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q45" s="77"/>
+      <c r="P45" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q45" s="107"/>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
       <c r="V45" s="61">
@@ -2774,11 +2735,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O46" s="28"/>
-      <c r="P46" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q46" s="77"/>
+      <c r="P46" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q46" s="107"/>
       <c r="R46" s="1"/>
       <c r="S46" s="1"/>
       <c r="V46" s="61">
@@ -2817,11 +2778,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O47" s="28"/>
-      <c r="P47" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q47" s="77"/>
+      <c r="P47" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q47" s="107"/>
       <c r="R47" s="1"/>
       <c r="S47" s="1"/>
       <c r="V47" s="61">
@@ -2860,11 +2821,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O48" s="28"/>
-      <c r="P48" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q48" s="77"/>
+      <c r="P48" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q48" s="107"/>
       <c r="R48" s="1"/>
       <c r="S48" s="1"/>
       <c r="V48" s="61">
@@ -2903,11 +2864,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O49" s="28"/>
-      <c r="P49" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q49" s="77"/>
+      <c r="P49" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q49" s="107"/>
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
       <c r="V49" s="61">
@@ -2946,11 +2907,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O50" s="28"/>
-      <c r="P50" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q50" s="77"/>
+      <c r="P50" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q50" s="107"/>
       <c r="R50" s="1"/>
       <c r="S50" s="1"/>
       <c r="V50" s="61">
@@ -2989,11 +2950,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O51" s="28"/>
-      <c r="P51" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q51" s="77"/>
+      <c r="P51" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q51" s="107"/>
       <c r="R51" s="1"/>
       <c r="S51" s="1"/>
       <c r="V51" s="61">
@@ -3032,11 +2993,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O52" s="28"/>
-      <c r="P52" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q52" s="77"/>
+      <c r="P52" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q52" s="107"/>
       <c r="R52" s="1"/>
       <c r="S52" s="1"/>
       <c r="V52" s="61">
@@ -3075,11 +3036,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O53" s="28"/>
-      <c r="P53" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q53" s="77"/>
+      <c r="P53" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q53" s="107"/>
       <c r="R53" s="1"/>
       <c r="S53" s="1"/>
       <c r="V53" s="61">
@@ -3118,11 +3079,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O54" s="28"/>
-      <c r="P54" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q54" s="77"/>
+      <c r="P54" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q54" s="107"/>
       <c r="R54" s="1"/>
       <c r="S54" s="1"/>
       <c r="V54" s="61">
@@ -3161,11 +3122,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O55" s="28"/>
-      <c r="P55" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q55" s="77"/>
+      <c r="P55" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q55" s="107"/>
       <c r="R55" s="1"/>
       <c r="S55" s="1"/>
       <c r="V55" s="61">
@@ -3204,11 +3165,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O56" s="28"/>
-      <c r="P56" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q56" s="77"/>
+      <c r="P56" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q56" s="107"/>
       <c r="R56" s="1"/>
       <c r="S56" s="1"/>
       <c r="V56" s="61">
@@ -3247,11 +3208,11 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="O57" s="28"/>
-      <c r="P57" s="76" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="Q57" s="77"/>
+      <c r="P57" s="106" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="Q57" s="107"/>
       <c r="R57" s="1"/>
       <c r="S57" s="1"/>
       <c r="V57" s="61">
@@ -3270,17 +3231,17 @@
       <c r="H58" s="1"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
-      <c r="L58" s="89" t="s">
+      <c r="L58" s="109" t="s">
         <v>29</v>
       </c>
-      <c r="M58" s="90"/>
-      <c r="N58" s="91"/>
+      <c r="M58" s="110"/>
+      <c r="N58" s="111"/>
       <c r="O58" s="7"/>
-      <c r="P58" s="97">
+      <c r="P58" s="82">
         <f>SUM(P38:P57)</f>
         <v>0</v>
       </c>
-      <c r="Q58" s="98"/>
+      <c r="Q58" s="83"/>
       <c r="S58" s="1"/>
     </row>
     <row r="59" spans="1:22" ht="7.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -3297,27 +3258,27 @@
     <row r="60" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
-      <c r="C60" s="93" t="str">
+      <c r="C60" s="112" t="str">
         <f>IF('Business Details'!B14&gt;0,'Business Details'!B14," ")</f>
         <v>Terms strictly 30 days net</v>
       </c>
-      <c r="D60" s="93"/>
-      <c r="E60" s="93"/>
-      <c r="F60" s="93"/>
-      <c r="G60" s="93"/>
-      <c r="H60" s="93"/>
-      <c r="I60" s="93"/>
-      <c r="L60" s="89" t="s">
+      <c r="D60" s="112"/>
+      <c r="E60" s="112"/>
+      <c r="F60" s="112"/>
+      <c r="G60" s="112"/>
+      <c r="H60" s="112"/>
+      <c r="I60" s="112"/>
+      <c r="L60" s="109" t="s">
         <v>30</v>
       </c>
-      <c r="M60" s="90"/>
-      <c r="N60" s="91"/>
+      <c r="M60" s="110"/>
+      <c r="N60" s="111"/>
       <c r="O60" s="7"/>
-      <c r="P60" s="97" t="str">
+      <c r="P60" s="82" t="str">
         <f>IF(N27=" "," ",IF(N27&gt;0,IF(LOOKUP(N27,'Invoice Database'!B:B,'Invoice Database'!E:E)&gt;0,LOOKUP(N27,'Invoice Database'!B:B,'Invoice Database'!E:E),0)))</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="Q60" s="98"/>
+      <c r="Q60" s="83"/>
       <c r="S60" s="1"/>
     </row>
     <row r="61" spans="1:22" ht="7.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -3334,27 +3295,27 @@
     <row r="62" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
-      <c r="C62" s="83" t="str">
+      <c r="C62" s="113" t="str">
         <f>IF('Business Details'!B15&gt;0,'Business Details'!B15," ")</f>
         <v xml:space="preserve">Overdue accounts charged at 2% per month </v>
       </c>
-      <c r="D62" s="83"/>
-      <c r="E62" s="83"/>
-      <c r="F62" s="83"/>
-      <c r="G62" s="83"/>
-      <c r="H62" s="83"/>
-      <c r="I62" s="83"/>
-      <c r="L62" s="89" t="s">
+      <c r="D62" s="113"/>
+      <c r="E62" s="113"/>
+      <c r="F62" s="113"/>
+      <c r="G62" s="113"/>
+      <c r="H62" s="113"/>
+      <c r="I62" s="113"/>
+      <c r="L62" s="109" t="s">
         <v>31</v>
       </c>
-      <c r="M62" s="90"/>
-      <c r="N62" s="91"/>
+      <c r="M62" s="110"/>
+      <c r="N62" s="111"/>
       <c r="O62" s="7"/>
-      <c r="P62" s="97">
+      <c r="P62" s="82">
         <f>IF(P58&lt;&gt;0,SUM(V38:V57)+P60*0.2,0)</f>
         <v>0</v>
       </c>
-      <c r="Q62" s="98"/>
+      <c r="Q62" s="83"/>
       <c r="S62" s="1"/>
     </row>
     <row r="63" spans="1:22" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -3371,28 +3332,28 @@
     <row r="64" spans="1:22" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
-      <c r="C64" s="93" t="str">
+      <c r="C64" s="112" t="str">
         <f>IF('Business Details'!B16&gt;0,'Business Details'!B16," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="D64" s="93"/>
-      <c r="E64" s="93"/>
-      <c r="F64" s="93"/>
-      <c r="G64" s="93"/>
-      <c r="H64" s="93"/>
-      <c r="I64" s="93"/>
-      <c r="L64" s="94" t="str">
+      <c r="D64" s="112"/>
+      <c r="E64" s="112"/>
+      <c r="F64" s="112"/>
+      <c r="G64" s="112"/>
+      <c r="H64" s="112"/>
+      <c r="I64" s="112"/>
+      <c r="L64" s="99" t="str">
         <f>IF(P64&lt;0,"Credit Amount","Amount Payable")</f>
         <v>Amount Payable</v>
       </c>
-      <c r="M64" s="95"/>
-      <c r="N64" s="96"/>
+      <c r="M64" s="100"/>
+      <c r="N64" s="101"/>
       <c r="O64" s="9"/>
-      <c r="P64" s="103">
+      <c r="P64" s="104">
         <f>SUM(P58:Q62)</f>
         <v>0</v>
       </c>
-      <c r="Q64" s="104"/>
+      <c r="Q64" s="105"/>
       <c r="S64" s="1"/>
     </row>
     <row r="65" spans="1:20" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
@@ -3409,24 +3370,24 @@
     <row r="66" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
-      <c r="C66" s="92" t="str">
+      <c r="C66" s="81" t="str">
         <f>IF('Business Details'!B17&gt;0,'Business Details'!B17," ")</f>
         <v>All goods remain the property of &lt;enter business name&gt; until paid for in full</v>
       </c>
-      <c r="D66" s="92"/>
-      <c r="E66" s="92"/>
-      <c r="F66" s="92"/>
-      <c r="G66" s="92"/>
-      <c r="H66" s="92"/>
-      <c r="I66" s="92"/>
-      <c r="J66" s="92"/>
-      <c r="K66" s="92"/>
-      <c r="L66" s="92"/>
-      <c r="M66" s="92"/>
-      <c r="N66" s="92"/>
-      <c r="O66" s="92"/>
-      <c r="P66" s="92"/>
-      <c r="Q66" s="92"/>
+      <c r="D66" s="81"/>
+      <c r="E66" s="81"/>
+      <c r="F66" s="81"/>
+      <c r="G66" s="81"/>
+      <c r="H66" s="81"/>
+      <c r="I66" s="81"/>
+      <c r="J66" s="81"/>
+      <c r="K66" s="81"/>
+      <c r="L66" s="81"/>
+      <c r="M66" s="81"/>
+      <c r="N66" s="81"/>
+      <c r="O66" s="81"/>
+      <c r="P66" s="81"/>
+      <c r="Q66" s="81"/>
       <c r="S66" s="1"/>
     </row>
     <row r="67" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.15">
@@ -3437,24 +3398,24 @@
     <row r="68" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
-      <c r="C68" s="92" t="str">
+      <c r="C68" s="81" t="str">
         <f>IF('Business Details'!B18&gt;0,'Business Details'!B18," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="D68" s="92"/>
-      <c r="E68" s="92"/>
-      <c r="F68" s="92"/>
-      <c r="G68" s="92"/>
-      <c r="H68" s="92"/>
-      <c r="I68" s="92"/>
-      <c r="J68" s="92"/>
-      <c r="K68" s="92"/>
-      <c r="L68" s="92"/>
-      <c r="M68" s="92"/>
-      <c r="N68" s="92"/>
-      <c r="O68" s="92"/>
-      <c r="P68" s="92"/>
-      <c r="Q68" s="92"/>
+      <c r="D68" s="81"/>
+      <c r="E68" s="81"/>
+      <c r="F68" s="81"/>
+      <c r="G68" s="81"/>
+      <c r="H68" s="81"/>
+      <c r="I68" s="81"/>
+      <c r="J68" s="81"/>
+      <c r="K68" s="81"/>
+      <c r="L68" s="81"/>
+      <c r="M68" s="81"/>
+      <c r="N68" s="81"/>
+      <c r="O68" s="81"/>
+      <c r="P68" s="81"/>
+      <c r="Q68" s="81"/>
       <c r="S68" s="1"/>
     </row>
     <row r="69" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3472,32 +3433,114 @@
       <c r="S69" s="1"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A70" s="88" t="s">
+      <c r="A70" s="108" t="s">
         <v>65</v>
       </c>
-      <c r="B70" s="88"/>
-      <c r="C70" s="88"/>
-      <c r="D70" s="88"/>
-      <c r="E70" s="88"/>
-      <c r="F70" s="88"/>
-      <c r="G70" s="88"/>
-      <c r="H70" s="88"/>
-      <c r="I70" s="88"/>
-      <c r="J70" s="88"/>
-      <c r="K70" s="88"/>
-      <c r="L70" s="88"/>
-      <c r="M70" s="88"/>
-      <c r="N70" s="88"/>
-      <c r="O70" s="88"/>
-      <c r="P70" s="88"/>
-      <c r="Q70" s="88"/>
-      <c r="R70" s="88"/>
-      <c r="S70" s="88"/>
+      <c r="B70" s="108"/>
+      <c r="C70" s="108"/>
+      <c r="D70" s="108"/>
+      <c r="E70" s="108"/>
+      <c r="F70" s="108"/>
+      <c r="G70" s="108"/>
+      <c r="H70" s="108"/>
+      <c r="I70" s="108"/>
+      <c r="J70" s="108"/>
+      <c r="K70" s="108"/>
+      <c r="L70" s="108"/>
+      <c r="M70" s="108"/>
+      <c r="N70" s="108"/>
+      <c r="O70" s="108"/>
+      <c r="P70" s="108"/>
+      <c r="Q70" s="108"/>
+      <c r="R70" s="108"/>
+      <c r="S70" s="108"/>
       <c r="T70" s="62"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="106">
+    <mergeCell ref="E49:H49"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="J13:P13"/>
+    <mergeCell ref="J14:P14"/>
+    <mergeCell ref="P45:Q45"/>
+    <mergeCell ref="P46:Q46"/>
+    <mergeCell ref="P47:Q47"/>
+    <mergeCell ref="P48:Q48"/>
+    <mergeCell ref="P41:Q41"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="P43:Q43"/>
+    <mergeCell ref="P44:Q44"/>
+    <mergeCell ref="P37:Q37"/>
+    <mergeCell ref="C31:G31"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="E37:H37"/>
+    <mergeCell ref="E45:H45"/>
+    <mergeCell ref="E43:H43"/>
+    <mergeCell ref="E44:H44"/>
+    <mergeCell ref="C30:G30"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="J6:P6"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C5:G6"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="A70:S70"/>
+    <mergeCell ref="E38:H38"/>
+    <mergeCell ref="E39:H39"/>
+    <mergeCell ref="E40:H40"/>
+    <mergeCell ref="E41:H41"/>
+    <mergeCell ref="E42:H42"/>
+    <mergeCell ref="L58:N58"/>
+    <mergeCell ref="L60:N60"/>
+    <mergeCell ref="L62:N62"/>
+    <mergeCell ref="E50:H50"/>
+    <mergeCell ref="E51:H51"/>
+    <mergeCell ref="E52:H52"/>
+    <mergeCell ref="E53:H53"/>
+    <mergeCell ref="E54:H54"/>
+    <mergeCell ref="E55:H55"/>
+    <mergeCell ref="E56:H56"/>
+    <mergeCell ref="P38:Q38"/>
+    <mergeCell ref="P39:Q39"/>
+    <mergeCell ref="P40:Q40"/>
+    <mergeCell ref="P57:Q57"/>
+    <mergeCell ref="C68:Q68"/>
+    <mergeCell ref="C60:I60"/>
+    <mergeCell ref="C62:I62"/>
+    <mergeCell ref="C64:I64"/>
+    <mergeCell ref="L64:N64"/>
+    <mergeCell ref="P60:Q60"/>
+    <mergeCell ref="J15:P15"/>
+    <mergeCell ref="J16:P16"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="J23:P23"/>
+    <mergeCell ref="J22:L22"/>
+    <mergeCell ref="N22:P22"/>
+    <mergeCell ref="J17:P17"/>
+    <mergeCell ref="J18:P18"/>
+    <mergeCell ref="J19:P19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="J29:L29"/>
+    <mergeCell ref="J31:L31"/>
+    <mergeCell ref="P62:Q62"/>
+    <mergeCell ref="P64:Q64"/>
+    <mergeCell ref="P53:Q53"/>
+    <mergeCell ref="P54:Q54"/>
+    <mergeCell ref="P55:Q55"/>
+    <mergeCell ref="P56:Q56"/>
+    <mergeCell ref="P49:Q49"/>
+    <mergeCell ref="P50:Q50"/>
+    <mergeCell ref="P51:Q51"/>
+    <mergeCell ref="P52:Q52"/>
     <mergeCell ref="E57:H57"/>
     <mergeCell ref="C27:G27"/>
     <mergeCell ref="C29:G29"/>
@@ -3522,88 +3565,6 @@
     <mergeCell ref="E46:H46"/>
     <mergeCell ref="E47:H47"/>
     <mergeCell ref="E48:H48"/>
-    <mergeCell ref="L64:N64"/>
-    <mergeCell ref="P60:Q60"/>
-    <mergeCell ref="J15:P15"/>
-    <mergeCell ref="J16:P16"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="J23:P23"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="N22:P22"/>
-    <mergeCell ref="J17:P17"/>
-    <mergeCell ref="J18:P18"/>
-    <mergeCell ref="J19:P19"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="J29:L29"/>
-    <mergeCell ref="J31:L31"/>
-    <mergeCell ref="P62:Q62"/>
-    <mergeCell ref="P64:Q64"/>
-    <mergeCell ref="P53:Q53"/>
-    <mergeCell ref="P54:Q54"/>
-    <mergeCell ref="P55:Q55"/>
-    <mergeCell ref="P56:Q56"/>
-    <mergeCell ref="P49:Q49"/>
-    <mergeCell ref="P50:Q50"/>
-    <mergeCell ref="P51:Q51"/>
-    <mergeCell ref="P52:Q52"/>
-    <mergeCell ref="A70:S70"/>
-    <mergeCell ref="E38:H38"/>
-    <mergeCell ref="E39:H39"/>
-    <mergeCell ref="E40:H40"/>
-    <mergeCell ref="E41:H41"/>
-    <mergeCell ref="E42:H42"/>
-    <mergeCell ref="L58:N58"/>
-    <mergeCell ref="L60:N60"/>
-    <mergeCell ref="L62:N62"/>
-    <mergeCell ref="E50:H50"/>
-    <mergeCell ref="E51:H51"/>
-    <mergeCell ref="E52:H52"/>
-    <mergeCell ref="E53:H53"/>
-    <mergeCell ref="E54:H54"/>
-    <mergeCell ref="E55:H55"/>
-    <mergeCell ref="E56:H56"/>
-    <mergeCell ref="P38:Q38"/>
-    <mergeCell ref="P39:Q39"/>
-    <mergeCell ref="P40:Q40"/>
-    <mergeCell ref="P57:Q57"/>
-    <mergeCell ref="C68:Q68"/>
-    <mergeCell ref="C60:I60"/>
-    <mergeCell ref="C62:I62"/>
-    <mergeCell ref="C64:I64"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="J6:P6"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C5:G6"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="E49:H49"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="J13:P13"/>
-    <mergeCell ref="J14:P14"/>
-    <mergeCell ref="P45:Q45"/>
-    <mergeCell ref="P46:Q46"/>
-    <mergeCell ref="P47:Q47"/>
-    <mergeCell ref="P48:Q48"/>
-    <mergeCell ref="P41:Q41"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="P43:Q43"/>
-    <mergeCell ref="P44:Q44"/>
-    <mergeCell ref="P37:Q37"/>
-    <mergeCell ref="C31:G31"/>
-    <mergeCell ref="C33:G33"/>
-    <mergeCell ref="C35:G35"/>
-    <mergeCell ref="E37:H37"/>
-    <mergeCell ref="E45:H45"/>
-    <mergeCell ref="E43:H43"/>
-    <mergeCell ref="E44:H44"/>
-    <mergeCell ref="C30:G30"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -3617,18 +3578,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AS1"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="39" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" style="40" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" style="41" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" style="40" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" style="42" customWidth="1"/>
-    <col min="6" max="45" width="8.5703125" style="40" customWidth="1"/>
-    <col min="46" max="16384" width="9.140625" style="43"/>
+    <col min="1" max="1" width="9.83203125" style="39" customWidth="1"/>
+    <col min="2" max="2" width="8.5" style="40" customWidth="1"/>
+    <col min="3" max="3" width="8.5" style="41" customWidth="1"/>
+    <col min="4" max="4" width="8.5" style="40" customWidth="1"/>
+    <col min="5" max="5" width="8.5" style="42" customWidth="1"/>
+    <col min="6" max="45" width="8.5" style="40" customWidth="1"/>
+    <col min="46" max="16384" width="9.1640625" style="43"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" s="38" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:45" s="38" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="60" t="s">
         <v>70</v>
       </c>
@@ -3777,20 +3738,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M101"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="47"/>
-    <col min="2" max="3" width="20.7109375" style="48" customWidth="1"/>
-    <col min="4" max="6" width="21.7109375" style="48" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" style="48" customWidth="1"/>
-    <col min="8" max="8" width="1.140625" style="48" customWidth="1"/>
-    <col min="9" max="9" width="20.7109375" style="48" customWidth="1"/>
-    <col min="10" max="12" width="21.7109375" style="48" customWidth="1"/>
-    <col min="13" max="13" width="9.7109375" style="48" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="48"/>
+    <col min="1" max="1" width="9.1640625" style="47"/>
+    <col min="2" max="3" width="20.6640625" style="48" customWidth="1"/>
+    <col min="4" max="6" width="21.6640625" style="48" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" style="48" customWidth="1"/>
+    <col min="8" max="8" width="1.1640625" style="48" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" style="48" customWidth="1"/>
+    <col min="10" max="12" width="21.6640625" style="48" customWidth="1"/>
+    <col min="13" max="13" width="9.6640625" style="48" customWidth="1"/>
+    <col min="14" max="16384" width="9.1640625" style="48"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="46" customFormat="1" ht="36" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" s="46" customFormat="1" ht="39" x14ac:dyDescent="0.15">
       <c r="A1" s="44" t="s">
         <v>42</v>
       </c>
@@ -3828,7 +3789,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="47">
         <v>101</v>
       </c>
@@ -3871,7 +3832,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B3" s="70" t="s">
         <v>77</v>
       </c>
@@ -3911,7 +3872,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B4" s="70" t="s">
         <v>77</v>
       </c>
@@ -3951,7 +3912,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B5" s="70" t="s">
         <v>77</v>
       </c>
@@ -3971,7 +3932,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B6" s="70" t="s">
         <v>77</v>
       </c>
@@ -3991,7 +3952,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B7" s="70" t="s">
         <v>77</v>
       </c>
@@ -4011,7 +3972,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B8" s="70" t="s">
         <v>77</v>
       </c>
@@ -4031,7 +3992,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B9" s="70" t="s">
         <v>77</v>
       </c>
@@ -4051,7 +4012,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B10" s="70" t="s">
         <v>77</v>
       </c>
@@ -4091,7 +4052,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B11" s="70" t="s">
         <v>77</v>
       </c>
@@ -4131,7 +4092,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B12" s="70" t="s">
         <v>77</v>
       </c>
@@ -4171,7 +4132,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B13" s="70" t="s">
         <v>77</v>
       </c>
@@ -4211,7 +4172,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B14" s="70" t="s">
         <v>77</v>
       </c>
@@ -4251,7 +4212,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B15" s="70" t="s">
         <v>77</v>
       </c>
@@ -4291,7 +4252,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B16" s="70" t="s">
         <v>77</v>
       </c>
@@ -4331,7 +4292,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B17" s="70" t="s">
         <v>77</v>
       </c>
@@ -4371,7 +4332,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B18" s="70" t="s">
         <v>77</v>
       </c>
@@ -4411,7 +4372,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B19" s="70" t="s">
         <v>77</v>
       </c>
@@ -4451,7 +4412,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B20" s="70" t="s">
         <v>77</v>
       </c>
@@ -4491,7 +4452,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B21" s="70" t="s">
         <v>77</v>
       </c>
@@ -4531,7 +4492,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B22" s="70" t="s">
         <v>77</v>
       </c>
@@ -4571,7 +4532,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B23" s="70" t="s">
         <v>77</v>
       </c>
@@ -4611,7 +4572,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B24" s="70" t="s">
         <v>77</v>
       </c>
@@ -4651,7 +4612,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B25" s="70" t="s">
         <v>77</v>
       </c>
@@ -4691,7 +4652,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B26" s="70" t="s">
         <v>77</v>
       </c>
@@ -4731,7 +4692,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B27" s="70" t="s">
         <v>77</v>
       </c>
@@ -4771,7 +4732,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B28" s="70" t="s">
         <v>77</v>
       </c>
@@ -4811,7 +4772,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B29" s="70" t="s">
         <v>77</v>
       </c>
@@ -4851,7 +4812,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B30" s="70" t="s">
         <v>77</v>
       </c>
@@ -4891,7 +4852,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B31" s="70" t="s">
         <v>77</v>
       </c>
@@ -4931,7 +4892,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B32" s="70" t="s">
         <v>77</v>
       </c>
@@ -4971,7 +4932,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B33" s="70" t="s">
         <v>77</v>
       </c>
@@ -5011,7 +4972,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B34" s="70" t="s">
         <v>77</v>
       </c>
@@ -5051,7 +5012,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B35" s="70" t="s">
         <v>77</v>
       </c>
@@ -5091,7 +5052,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B36" s="70" t="s">
         <v>77</v>
       </c>
@@ -5131,7 +5092,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B37" s="70" t="s">
         <v>77</v>
       </c>
@@ -5171,7 +5132,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B38" s="70" t="s">
         <v>77</v>
       </c>
@@ -5211,7 +5172,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B39" s="70" t="s">
         <v>77</v>
       </c>
@@ -5251,7 +5212,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B40" s="70" t="s">
         <v>77</v>
       </c>
@@ -5291,7 +5252,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B41" s="70" t="s">
         <v>77</v>
       </c>
@@ -5331,7 +5292,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B42" s="70" t="s">
         <v>77</v>
       </c>
@@ -5371,7 +5332,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B43" s="70" t="s">
         <v>77</v>
       </c>
@@ -5411,7 +5372,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B44" s="70" t="s">
         <v>77</v>
       </c>
@@ -5451,7 +5412,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B45" s="70" t="s">
         <v>77</v>
       </c>
@@ -5491,7 +5452,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B46" s="70" t="s">
         <v>77</v>
       </c>
@@ -5531,7 +5492,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B47" s="70" t="s">
         <v>77</v>
       </c>
@@ -5571,7 +5532,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B48" s="70" t="s">
         <v>77</v>
       </c>
@@ -5611,7 +5572,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B49" s="70" t="s">
         <v>77</v>
       </c>
@@ -5651,7 +5612,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B50" s="70" t="s">
         <v>77</v>
       </c>
@@ -5691,7 +5652,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B51" s="70" t="s">
         <v>77</v>
       </c>
@@ -5731,7 +5692,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B52" s="70" t="s">
         <v>77</v>
       </c>
@@ -5771,7 +5732,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B53" s="70" t="s">
         <v>77</v>
       </c>
@@ -5811,7 +5772,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B54" s="70" t="s">
         <v>77</v>
       </c>
@@ -5851,7 +5812,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B55" s="70" t="s">
         <v>77</v>
       </c>
@@ -5891,7 +5852,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B56" s="70" t="s">
         <v>77</v>
       </c>
@@ -5931,7 +5892,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B57" s="70" t="s">
         <v>77</v>
       </c>
@@ -5971,7 +5932,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B58" s="70" t="s">
         <v>77</v>
       </c>
@@ -6011,7 +5972,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="59" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B59" s="70" t="s">
         <v>77</v>
       </c>
@@ -6051,7 +6012,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B60" s="70" t="s">
         <v>77</v>
       </c>
@@ -6091,7 +6052,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B61" s="70" t="s">
         <v>77</v>
       </c>
@@ -6131,7 +6092,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B62" s="70" t="s">
         <v>77</v>
       </c>
@@ -6171,7 +6132,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B63" s="70" t="s">
         <v>77</v>
       </c>
@@ -6211,7 +6172,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B64" s="70" t="s">
         <v>77</v>
       </c>
@@ -6251,7 +6212,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B65" s="70" t="s">
         <v>77</v>
       </c>
@@ -6291,7 +6252,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B66" s="70" t="s">
         <v>77</v>
       </c>
@@ -6331,7 +6292,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B67" s="70" t="s">
         <v>77</v>
       </c>
@@ -6371,7 +6332,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B68" s="70" t="s">
         <v>77</v>
       </c>
@@ -6411,7 +6372,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B69" s="70" t="s">
         <v>77</v>
       </c>
@@ -6451,7 +6412,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B70" s="70" t="s">
         <v>77</v>
       </c>
@@ -6491,7 +6452,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B71" s="70" t="s">
         <v>77</v>
       </c>
@@ -6531,7 +6492,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B72" s="70" t="s">
         <v>77</v>
       </c>
@@ -6571,7 +6532,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B73" s="70" t="s">
         <v>77</v>
       </c>
@@ -6611,7 +6572,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B74" s="70" t="s">
         <v>77</v>
       </c>
@@ -6651,7 +6612,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B75" s="70" t="s">
         <v>77</v>
       </c>
@@ -6691,7 +6652,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B76" s="70" t="s">
         <v>77</v>
       </c>
@@ -6731,7 +6692,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B77" s="70" t="s">
         <v>77</v>
       </c>
@@ -6771,7 +6732,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B78" s="70" t="s">
         <v>77</v>
       </c>
@@ -6811,7 +6772,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B79" s="70" t="s">
         <v>77</v>
       </c>
@@ -6851,7 +6812,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B80" s="70" t="s">
         <v>77</v>
       </c>
@@ -6891,7 +6852,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B81" s="70" t="s">
         <v>77</v>
       </c>
@@ -6931,7 +6892,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B82" s="70" t="s">
         <v>77</v>
       </c>
@@ -6971,7 +6932,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B83" s="70" t="s">
         <v>77</v>
       </c>
@@ -7011,7 +6972,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B84" s="70" t="s">
         <v>77</v>
       </c>
@@ -7051,7 +7012,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B85" s="70" t="s">
         <v>77</v>
       </c>
@@ -7091,7 +7052,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B86" s="70" t="s">
         <v>77</v>
       </c>
@@ -7131,7 +7092,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B87" s="70" t="s">
         <v>77</v>
       </c>
@@ -7171,7 +7132,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B88" s="70" t="s">
         <v>77</v>
       </c>
@@ -7211,7 +7172,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B89" s="70" t="s">
         <v>77</v>
       </c>
@@ -7251,7 +7212,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B90" s="70" t="s">
         <v>77</v>
       </c>
@@ -7291,7 +7252,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B91" s="70" t="s">
         <v>77</v>
       </c>
@@ -7331,7 +7292,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B92" s="70" t="s">
         <v>77</v>
       </c>
@@ -7371,7 +7332,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B93" s="70" t="s">
         <v>77</v>
       </c>
@@ -7411,7 +7372,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B94" s="70" t="s">
         <v>77</v>
       </c>
@@ -7451,7 +7412,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B95" s="70" t="s">
         <v>77</v>
       </c>
@@ -7491,7 +7452,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B96" s="70" t="s">
         <v>77</v>
       </c>
@@ -7531,7 +7492,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B97" s="70" t="s">
         <v>77</v>
       </c>
@@ -7571,7 +7532,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B98" s="70" t="s">
         <v>77</v>
       </c>
@@ -7611,7 +7572,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B99" s="70" t="s">
         <v>77</v>
       </c>
@@ -7651,7 +7612,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:13" ht="13" x14ac:dyDescent="0.15">
       <c r="B100" s="70" t="s">
         <v>77</v>
       </c>
@@ -7691,7 +7652,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:13" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:13" ht="14" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A101" s="49"/>
       <c r="B101" s="49" t="s">
         <v>77</v>
@@ -7745,19 +7706,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H99"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="53" customWidth="1"/>
-    <col min="2" max="2" width="29.140625" style="54" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="55" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="56" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="53" customWidth="1"/>
+    <col min="2" max="2" width="29.1640625" style="54" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="55" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" style="56" customWidth="1"/>
     <col min="5" max="5" width="1" style="54" customWidth="1"/>
-    <col min="6" max="7" width="10.7109375" style="55" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" style="56" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="54"/>
+    <col min="6" max="7" width="10.6640625" style="55" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="56" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="54"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="48" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="48" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="44" t="s">
         <v>49</v>
       </c>
@@ -7780,7 +7741,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="53">
         <v>1001</v>
       </c>
@@ -7796,7 +7757,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D3" s="56">
         <v>20</v>
       </c>
@@ -7809,7 +7770,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D4" s="56">
         <v>20</v>
       </c>
@@ -7822,7 +7783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D5" s="56">
         <v>20</v>
       </c>
@@ -7835,7 +7796,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D6" s="56">
         <v>20</v>
       </c>
@@ -7845,7 +7806,7 @@
       </c>
       <c r="H6" s="64"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D7" s="56">
         <v>20</v>
       </c>
@@ -7855,7 +7816,7 @@
       </c>
       <c r="H7" s="64"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D8" s="56">
         <v>20</v>
       </c>
@@ -7865,7 +7826,7 @@
       </c>
       <c r="H8" s="64"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D9" s="56">
         <v>20</v>
       </c>
@@ -7875,7 +7836,7 @@
       </c>
       <c r="H9" s="64"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D10" s="56">
         <v>20</v>
       </c>
@@ -7885,7 +7846,7 @@
       </c>
       <c r="H10" s="64"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D11" s="56">
         <v>20</v>
       </c>
@@ -7895,7 +7856,7 @@
       </c>
       <c r="H11" s="64"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D12" s="56">
         <v>20</v>
       </c>
@@ -7905,7 +7866,7 @@
       </c>
       <c r="H12" s="64"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D13" s="56">
         <v>20</v>
       </c>
@@ -7915,7 +7876,7 @@
       </c>
       <c r="H13" s="64"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D14" s="56">
         <v>20</v>
       </c>
@@ -7925,7 +7886,7 @@
       </c>
       <c r="H14" s="64"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D15" s="56">
         <v>20</v>
       </c>
@@ -7935,7 +7896,7 @@
       </c>
       <c r="H15" s="64"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D16" s="56">
         <v>20</v>
       </c>
@@ -7945,7 +7906,7 @@
       </c>
       <c r="H16" s="64"/>
     </row>
-    <row r="17" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D17" s="56">
         <v>20</v>
       </c>
@@ -7955,7 +7916,7 @@
       </c>
       <c r="H17" s="64"/>
     </row>
-    <row r="18" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D18" s="56">
         <v>20</v>
       </c>
@@ -7965,7 +7926,7 @@
       </c>
       <c r="H18" s="64"/>
     </row>
-    <row r="19" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D19" s="56">
         <v>20</v>
       </c>
@@ -7975,7 +7936,7 @@
       </c>
       <c r="H19" s="64"/>
     </row>
-    <row r="20" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D20" s="56">
         <v>20</v>
       </c>
@@ -7985,7 +7946,7 @@
       </c>
       <c r="H20" s="64"/>
     </row>
-    <row r="21" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D21" s="56">
         <v>20</v>
       </c>
@@ -7995,7 +7956,7 @@
       </c>
       <c r="H21" s="64"/>
     </row>
-    <row r="22" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D22" s="56">
         <v>20</v>
       </c>
@@ -8005,7 +7966,7 @@
       </c>
       <c r="H22" s="64"/>
     </row>
-    <row r="23" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D23" s="56">
         <v>20</v>
       </c>
@@ -8015,7 +7976,7 @@
       </c>
       <c r="H23" s="64"/>
     </row>
-    <row r="24" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D24" s="56">
         <v>20</v>
       </c>
@@ -8025,7 +7986,7 @@
       </c>
       <c r="H24" s="64"/>
     </row>
-    <row r="25" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D25" s="56">
         <v>20</v>
       </c>
@@ -8035,7 +7996,7 @@
       </c>
       <c r="H25" s="64"/>
     </row>
-    <row r="26" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D26" s="56">
         <v>20</v>
       </c>
@@ -8045,7 +8006,7 @@
       </c>
       <c r="H26" s="64"/>
     </row>
-    <row r="27" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D27" s="56">
         <v>20</v>
       </c>
@@ -8055,7 +8016,7 @@
       </c>
       <c r="H27" s="64"/>
     </row>
-    <row r="28" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D28" s="56">
         <v>20</v>
       </c>
@@ -8065,7 +8026,7 @@
       </c>
       <c r="H28" s="64"/>
     </row>
-    <row r="29" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D29" s="56">
         <v>20</v>
       </c>
@@ -8075,7 +8036,7 @@
       </c>
       <c r="H29" s="64"/>
     </row>
-    <row r="30" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D30" s="56">
         <v>20</v>
       </c>
@@ -8085,7 +8046,7 @@
       </c>
       <c r="H30" s="64"/>
     </row>
-    <row r="31" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D31" s="56">
         <v>20</v>
       </c>
@@ -8095,7 +8056,7 @@
       </c>
       <c r="H31" s="64"/>
     </row>
-    <row r="32" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D32" s="56">
         <v>20</v>
       </c>
@@ -8105,7 +8066,7 @@
       </c>
       <c r="H32" s="64"/>
     </row>
-    <row r="33" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D33" s="56">
         <v>20</v>
       </c>
@@ -8115,7 +8076,7 @@
       </c>
       <c r="H33" s="64"/>
     </row>
-    <row r="34" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D34" s="56">
         <v>20</v>
       </c>
@@ -8125,7 +8086,7 @@
       </c>
       <c r="H34" s="64"/>
     </row>
-    <row r="35" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D35" s="56">
         <v>20</v>
       </c>
@@ -8135,7 +8096,7 @@
       </c>
       <c r="H35" s="64"/>
     </row>
-    <row r="36" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D36" s="56">
         <v>20</v>
       </c>
@@ -8145,7 +8106,7 @@
       </c>
       <c r="H36" s="64"/>
     </row>
-    <row r="37" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D37" s="56">
         <v>20</v>
       </c>
@@ -8155,7 +8116,7 @@
       </c>
       <c r="H37" s="64"/>
     </row>
-    <row r="38" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D38" s="56">
         <v>20</v>
       </c>
@@ -8165,7 +8126,7 @@
       </c>
       <c r="H38" s="64"/>
     </row>
-    <row r="39" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D39" s="56">
         <v>20</v>
       </c>
@@ -8175,7 +8136,7 @@
       </c>
       <c r="H39" s="64"/>
     </row>
-    <row r="40" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D40" s="56">
         <v>20</v>
       </c>
@@ -8185,7 +8146,7 @@
       </c>
       <c r="H40" s="64"/>
     </row>
-    <row r="41" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D41" s="56">
         <v>20</v>
       </c>
@@ -8195,7 +8156,7 @@
       </c>
       <c r="H41" s="64"/>
     </row>
-    <row r="42" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D42" s="56">
         <v>20</v>
       </c>
@@ -8205,7 +8166,7 @@
       </c>
       <c r="H42" s="64"/>
     </row>
-    <row r="43" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D43" s="56">
         <v>20</v>
       </c>
@@ -8215,7 +8176,7 @@
       </c>
       <c r="H43" s="64"/>
     </row>
-    <row r="44" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D44" s="56">
         <v>20</v>
       </c>
@@ -8225,7 +8186,7 @@
       </c>
       <c r="H44" s="64"/>
     </row>
-    <row r="45" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D45" s="56">
         <v>20</v>
       </c>
@@ -8235,7 +8196,7 @@
       </c>
       <c r="H45" s="64"/>
     </row>
-    <row r="46" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D46" s="56">
         <v>20</v>
       </c>
@@ -8245,7 +8206,7 @@
       </c>
       <c r="H46" s="64"/>
     </row>
-    <row r="47" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D47" s="56">
         <v>20</v>
       </c>
@@ -8255,7 +8216,7 @@
       </c>
       <c r="H47" s="64"/>
     </row>
-    <row r="48" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D48" s="56">
         <v>20</v>
       </c>
@@ -8265,7 +8226,7 @@
       </c>
       <c r="H48" s="64"/>
     </row>
-    <row r="49" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D49" s="56">
         <v>20</v>
       </c>
@@ -8275,7 +8236,7 @@
       </c>
       <c r="H49" s="64"/>
     </row>
-    <row r="50" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D50" s="56">
         <v>20</v>
       </c>
@@ -8285,7 +8246,7 @@
       </c>
       <c r="H50" s="64"/>
     </row>
-    <row r="51" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D51" s="56">
         <v>20</v>
       </c>
@@ -8295,7 +8256,7 @@
       </c>
       <c r="H51" s="64"/>
     </row>
-    <row r="52" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D52" s="56">
         <v>20</v>
       </c>
@@ -8305,7 +8266,7 @@
       </c>
       <c r="H52" s="64"/>
     </row>
-    <row r="53" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D53" s="56">
         <v>20</v>
       </c>
@@ -8315,7 +8276,7 @@
       </c>
       <c r="H53" s="64"/>
     </row>
-    <row r="54" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D54" s="56">
         <v>20</v>
       </c>
@@ -8325,7 +8286,7 @@
       </c>
       <c r="H54" s="64"/>
     </row>
-    <row r="55" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D55" s="56">
         <v>20</v>
       </c>
@@ -8335,7 +8296,7 @@
       </c>
       <c r="H55" s="64"/>
     </row>
-    <row r="56" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D56" s="56">
         <v>20</v>
       </c>
@@ -8345,7 +8306,7 @@
       </c>
       <c r="H56" s="64"/>
     </row>
-    <row r="57" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D57" s="56">
         <v>20</v>
       </c>
@@ -8355,7 +8316,7 @@
       </c>
       <c r="H57" s="64"/>
     </row>
-    <row r="58" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D58" s="56">
         <v>20</v>
       </c>
@@ -8365,7 +8326,7 @@
       </c>
       <c r="H58" s="64"/>
     </row>
-    <row r="59" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D59" s="56">
         <v>20</v>
       </c>
@@ -8375,7 +8336,7 @@
       </c>
       <c r="H59" s="64"/>
     </row>
-    <row r="60" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D60" s="56">
         <v>20</v>
       </c>
@@ -8385,7 +8346,7 @@
       </c>
       <c r="H60" s="64"/>
     </row>
-    <row r="61" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D61" s="56">
         <v>20</v>
       </c>
@@ -8395,7 +8356,7 @@
       </c>
       <c r="H61" s="64"/>
     </row>
-    <row r="62" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D62" s="56">
         <v>20</v>
       </c>
@@ -8405,7 +8366,7 @@
       </c>
       <c r="H62" s="64"/>
     </row>
-    <row r="63" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D63" s="56">
         <v>20</v>
       </c>
@@ -8415,7 +8376,7 @@
       </c>
       <c r="H63" s="64"/>
     </row>
-    <row r="64" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D64" s="56">
         <v>20</v>
       </c>
@@ -8425,7 +8386,7 @@
       </c>
       <c r="H64" s="64"/>
     </row>
-    <row r="65" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D65" s="56">
         <v>20</v>
       </c>
@@ -8435,7 +8396,7 @@
       </c>
       <c r="H65" s="64"/>
     </row>
-    <row r="66" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D66" s="56">
         <v>20</v>
       </c>
@@ -8445,7 +8406,7 @@
       </c>
       <c r="H66" s="64"/>
     </row>
-    <row r="67" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D67" s="56">
         <v>20</v>
       </c>
@@ -8455,7 +8416,7 @@
       </c>
       <c r="H67" s="64"/>
     </row>
-    <row r="68" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D68" s="56">
         <v>20</v>
       </c>
@@ -8465,7 +8426,7 @@
       </c>
       <c r="H68" s="64"/>
     </row>
-    <row r="69" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D69" s="56">
         <v>20</v>
       </c>
@@ -8475,7 +8436,7 @@
       </c>
       <c r="H69" s="64"/>
     </row>
-    <row r="70" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D70" s="56">
         <v>20</v>
       </c>
@@ -8485,7 +8446,7 @@
       </c>
       <c r="H70" s="64"/>
     </row>
-    <row r="71" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D71" s="56">
         <v>20</v>
       </c>
@@ -8495,7 +8456,7 @@
       </c>
       <c r="H71" s="64"/>
     </row>
-    <row r="72" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D72" s="56">
         <v>20</v>
       </c>
@@ -8505,7 +8466,7 @@
       </c>
       <c r="H72" s="64"/>
     </row>
-    <row r="73" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D73" s="56">
         <v>20</v>
       </c>
@@ -8515,7 +8476,7 @@
       </c>
       <c r="H73" s="64"/>
     </row>
-    <row r="74" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D74" s="56">
         <v>20</v>
       </c>
@@ -8525,7 +8486,7 @@
       </c>
       <c r="H74" s="64"/>
     </row>
-    <row r="75" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D75" s="56">
         <v>20</v>
       </c>
@@ -8535,7 +8496,7 @@
       </c>
       <c r="H75" s="64"/>
     </row>
-    <row r="76" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D76" s="56">
         <v>20</v>
       </c>
@@ -8545,7 +8506,7 @@
       </c>
       <c r="H76" s="64"/>
     </row>
-    <row r="77" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D77" s="56">
         <v>20</v>
       </c>
@@ -8555,7 +8516,7 @@
       </c>
       <c r="H77" s="64"/>
     </row>
-    <row r="78" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D78" s="56">
         <v>20</v>
       </c>
@@ -8565,7 +8526,7 @@
       </c>
       <c r="H78" s="64"/>
     </row>
-    <row r="79" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D79" s="56">
         <v>20</v>
       </c>
@@ -8575,7 +8536,7 @@
       </c>
       <c r="H79" s="64"/>
     </row>
-    <row r="80" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D80" s="56">
         <v>20</v>
       </c>
@@ -8585,7 +8546,7 @@
       </c>
       <c r="H80" s="64"/>
     </row>
-    <row r="81" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="81" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D81" s="56">
         <v>20</v>
       </c>
@@ -8595,7 +8556,7 @@
       </c>
       <c r="H81" s="64"/>
     </row>
-    <row r="82" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="82" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D82" s="56">
         <v>20</v>
       </c>
@@ -8605,7 +8566,7 @@
       </c>
       <c r="H82" s="64"/>
     </row>
-    <row r="83" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D83" s="56">
         <v>20</v>
       </c>
@@ -8615,7 +8576,7 @@
       </c>
       <c r="H83" s="64"/>
     </row>
-    <row r="84" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="84" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D84" s="56">
         <v>20</v>
       </c>
@@ -8625,7 +8586,7 @@
       </c>
       <c r="H84" s="64"/>
     </row>
-    <row r="85" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="85" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D85" s="56">
         <v>20</v>
       </c>
@@ -8635,7 +8596,7 @@
       </c>
       <c r="H85" s="64"/>
     </row>
-    <row r="86" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="86" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D86" s="56">
         <v>20</v>
       </c>
@@ -8645,7 +8606,7 @@
       </c>
       <c r="H86" s="64"/>
     </row>
-    <row r="87" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="87" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D87" s="56">
         <v>20</v>
       </c>
@@ -8655,7 +8616,7 @@
       </c>
       <c r="H87" s="64"/>
     </row>
-    <row r="88" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D88" s="56">
         <v>20</v>
       </c>
@@ -8665,7 +8626,7 @@
       </c>
       <c r="H88" s="64"/>
     </row>
-    <row r="89" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="89" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D89" s="56">
         <v>20</v>
       </c>
@@ -8675,7 +8636,7 @@
       </c>
       <c r="H89" s="64"/>
     </row>
-    <row r="90" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="90" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D90" s="56">
         <v>20</v>
       </c>
@@ -8685,7 +8646,7 @@
       </c>
       <c r="H90" s="64"/>
     </row>
-    <row r="91" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="91" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D91" s="56">
         <v>20</v>
       </c>
@@ -8695,7 +8656,7 @@
       </c>
       <c r="H91" s="64"/>
     </row>
-    <row r="92" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="92" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D92" s="56">
         <v>20</v>
       </c>
@@ -8705,7 +8666,7 @@
       </c>
       <c r="H92" s="64"/>
     </row>
-    <row r="93" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="93" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D93" s="56">
         <v>20</v>
       </c>
@@ -8715,7 +8676,7 @@
       </c>
       <c r="H93" s="64"/>
     </row>
-    <row r="94" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="94" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D94" s="56">
         <v>20</v>
       </c>
@@ -8725,7 +8686,7 @@
       </c>
       <c r="H94" s="64"/>
     </row>
-    <row r="95" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="95" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D95" s="56">
         <v>20</v>
       </c>
@@ -8735,7 +8696,7 @@
       </c>
       <c r="H95" s="64"/>
     </row>
-    <row r="96" spans="4:8" x14ac:dyDescent="0.2">
+    <row r="96" spans="4:8" x14ac:dyDescent="0.15">
       <c r="D96" s="56">
         <v>20</v>
       </c>
@@ -8745,7 +8706,7 @@
       </c>
       <c r="H96" s="64"/>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D97" s="56">
         <v>20</v>
       </c>
@@ -8755,7 +8716,7 @@
       </c>
       <c r="H97" s="64"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.15">
       <c r="D98" s="56">
         <v>20</v>
       </c>
@@ -8765,7 +8726,7 @@
       </c>
       <c r="H98" s="64"/>
     </row>
-    <row r="99" spans="1:8" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" ht="13" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A99" s="57"/>
       <c r="B99" s="58"/>
       <c r="C99" s="59"/>
@@ -8790,23 +8751,23 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" style="17" customWidth="1"/>
-    <col min="2" max="2" width="43.85546875" style="17" customWidth="1"/>
-    <col min="3" max="3" width="2.7109375" style="17" customWidth="1"/>
-    <col min="4" max="6" width="9.140625" style="17"/>
-    <col min="7" max="7" width="12.140625" style="17" customWidth="1"/>
-    <col min="8" max="8" width="2.7109375" style="17" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="17"/>
+    <col min="1" max="1" width="23.83203125" style="17" customWidth="1"/>
+    <col min="2" max="2" width="43.83203125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="2.6640625" style="17" customWidth="1"/>
+    <col min="4" max="6" width="9.1640625" style="17"/>
+    <col min="7" max="7" width="12.1640625" style="17" customWidth="1"/>
+    <col min="8" max="8" width="2.6640625" style="17" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="17"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A1" s="21"/>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A2" s="22" t="s">
         <v>46</v>
       </c>
@@ -8816,7 +8777,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="22" t="s">
         <v>0</v>
       </c>
@@ -8828,7 +8789,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A4" s="22" t="s">
         <v>1</v>
       </c>
@@ -8838,7 +8799,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A5" s="22" t="s">
         <v>2</v>
       </c>
@@ -8848,7 +8809,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A6" s="22" t="s">
         <v>3</v>
       </c>
@@ -8858,35 +8819,35 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="22" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="23"/>
       <c r="C7" s="21"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="22" t="s">
         <v>39</v>
       </c>
       <c r="B8" s="24"/>
       <c r="C8" s="21"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A9" s="22" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="21"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A10" s="22" t="s">
         <v>40</v>
       </c>
       <c r="B10" s="30"/>
       <c r="C10" s="21"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A11" s="69" t="s">
         <v>81</v>
       </c>
@@ -8898,14 +8859,14 @@
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A12" s="22" t="s">
         <v>13</v>
       </c>
       <c r="B12" s="72"/>
       <c r="C12" s="21"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A13" s="22" t="s">
         <v>14</v>
       </c>
@@ -8914,7 +8875,7 @@
       </c>
       <c r="C13" s="21"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A14" s="22" t="s">
         <v>43</v>
       </c>
@@ -8923,7 +8884,7 @@
       </c>
       <c r="C14" s="21"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A15" s="22" t="s">
         <v>44</v>
       </c>
@@ -8932,7 +8893,7 @@
       </c>
       <c r="C15" s="21"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A16" s="22" t="s">
         <v>45</v>
       </c>
@@ -8944,7 +8905,7 @@
       <c r="G16" s="21"/>
       <c r="H16" s="21"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A17" s="22" t="s">
         <v>47</v>
       </c>
@@ -8959,7 +8920,7 @@
       <c r="G17" s="124"/>
       <c r="H17" s="21"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A18" s="22" t="s">
         <v>48</v>
       </c>
@@ -8971,7 +8932,7 @@
       <c r="G18" s="124"/>
       <c r="H18" s="21"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A19" s="21"/>
       <c r="B19" s="21"/>
       <c r="C19" s="21"/>

</xml_diff>